<commit_message>
data: atualizacao do painel (via botao)
</commit_message>
<xml_diff>
--- a/franquias/pwr_reports/KEYS Service Main Service Exceptions - Franquias (Stores)(2026-08-03 - 2026-08-09).xlsx
+++ b/franquias/pwr_reports/KEYS Service Main Service Exceptions - Franquias (Stores)(2026-08-03 - 2026-08-09).xlsx
@@ -908,51 +908,48 @@
     <t>187</t>
   </si>
   <si>
-    <t>155</t>
-  </si>
-  <si>
-    <t>R$ 41.956,98</t>
-  </si>
-  <si>
-    <t>431.5</t>
-  </si>
-  <si>
-    <t>261.2</t>
-  </si>
-  <si>
-    <t>5.71</t>
-  </si>
-  <si>
-    <t>19.7</t>
-  </si>
-  <si>
-    <t>7.3</t>
+    <t>121</t>
+  </si>
+  <si>
+    <t>R$ 42.334,49</t>
+  </si>
+  <si>
+    <t>448.4</t>
+  </si>
+  <si>
+    <t>273.9</t>
+  </si>
+  <si>
+    <t>5.76</t>
+  </si>
+  <si>
+    <t>19.8</t>
+  </si>
+  <si>
+    <t>7.4</t>
   </si>
   <si>
     <t>6.7</t>
   </si>
   <si>
-    <t>38.3%</t>
-  </si>
-  <si>
-    <t>19.2%</t>
+    <t>37.4%</t>
+  </si>
+  <si>
+    <t>19.1%</t>
   </si>
   <si>
     <t>2.2%</t>
   </si>
   <si>
-    <t>0.3%</t>
-  </si>
-  <si>
-    <t>5.6%</t>
+    <t>0.2%</t>
+  </si>
+  <si>
+    <t>5.5%</t>
   </si>
   <si>
     <t>1.3%</t>
   </si>
   <si>
-    <t>0.2%</t>
-  </si>
-  <si>
     <t>6.8%</t>
   </si>
   <si>
@@ -962,40 +959,40 @@
     <t>4.3%</t>
   </si>
   <si>
-    <t>10688.0</t>
-  </si>
-  <si>
-    <t>8683.0</t>
-  </si>
-  <si>
-    <t>976.0</t>
-  </si>
-  <si>
-    <t>113.0</t>
-  </si>
-  <si>
-    <t>2510.0</t>
-  </si>
-  <si>
-    <t>577.0</t>
-  </si>
-  <si>
-    <t>96.0</t>
-  </si>
-  <si>
-    <t>3088.0</t>
-  </si>
-  <si>
-    <t>1252.0</t>
-  </si>
-  <si>
-    <t>1944.0</t>
+    <t>11118.0</t>
+  </si>
+  <si>
+    <t>9056.0</t>
+  </si>
+  <si>
+    <t>1033.0</t>
+  </si>
+  <si>
+    <t>117.0</t>
+  </si>
+  <si>
+    <t>2590.0</t>
+  </si>
+  <si>
+    <t>598.0</t>
+  </si>
+  <si>
+    <t>99.0</t>
+  </si>
+  <si>
+    <t>3214.0</t>
+  </si>
+  <si>
+    <t>1312.0</t>
+  </si>
+  <si>
+    <t>2019.0</t>
   </si>
   <si>
     <t>0.5%</t>
   </si>
   <si>
-    <t>245.0</t>
+    <t>253.0</t>
   </si>
   <si>
     <t>1</t>
@@ -2246,7 +2243,7 @@
         <v>19521</v>
       </c>
       <c r="B6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C6" s="4">
         <v>51</v>
@@ -2277,7 +2274,7 @@
       </c>
       <c r="L6" s="4"/>
       <c r="M6" s="5">
-        <v>86064.42833333333</v>
+        <v>73769.509999999995</v>
       </c>
       <c r="N6" s="6">
         <v>743</v>
@@ -3758,7 +3755,7 @@
         <v>19546</v>
       </c>
       <c r="B16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C16" s="4">
         <v>51</v>
@@ -3789,70 +3786,70 @@
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="5">
-        <v>43241.251666666671</v>
+        <v>45140.139999999999</v>
       </c>
       <c r="N16" s="6">
-        <v>406</v>
+        <v>493</v>
       </c>
       <c r="O16" s="6">
-        <v>222</v>
+        <v>267</v>
       </c>
       <c r="P16" s="7">
-        <v>3.8390573232323231</v>
+        <v>3.9391078838174276</v>
       </c>
       <c r="Q16" s="8">
-        <v>18.929109954751134</v>
+        <v>19.007268045112781</v>
       </c>
       <c r="R16" s="8">
-        <v>8.2676557077625574</v>
+        <v>8.2512624999999993</v>
       </c>
       <c r="S16" s="8">
         <v>7</v>
       </c>
       <c r="T16" s="9">
-        <v>0.34841628959276016</v>
+        <v>0.32330827067669171</v>
       </c>
       <c r="U16" s="9">
-        <v>0.16666666666666666</v>
+        <v>0.14606741573033707</v>
       </c>
       <c r="V16" s="9">
-        <v>0.018018018018018018</v>
+        <v>0.018726591760299626</v>
       </c>
       <c r="W16" s="9">
         <v>0</v>
       </c>
       <c r="X16" s="9">
-        <v>0.11261261261261261</v>
+        <v>0.10112359550561797</v>
       </c>
       <c r="Y16" s="9">
-        <v>0.0090090090090090089</v>
+        <v>0.0074906367041198503</v>
       </c>
       <c r="Z16" s="9">
         <v>0</v>
       </c>
       <c r="AA16" s="9">
-        <v>0.018018018018018018</v>
+        <v>0.018726591760299626</v>
       </c>
       <c r="AB16" s="9">
-        <v>0.0045045045045045045</v>
+        <v>0.0037453183520599251</v>
       </c>
       <c r="AC16" s="9">
-        <v>0.036036036036036036</v>
+        <v>0.029962546816479401</v>
       </c>
       <c r="AD16" s="6">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AE16" s="6">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="AF16" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG16" s="6">
         <v>0</v>
       </c>
       <c r="AH16" s="6">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="AI16" s="6">
         <v>2</v>
@@ -3861,7 +3858,7 @@
         <v>0</v>
       </c>
       <c r="AK16" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL16" s="6">
         <v>1</v>
@@ -4072,7 +4069,7 @@
         <v>19550</v>
       </c>
       <c r="B18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C18" s="4">
         <v>51</v>
@@ -4103,34 +4100,34 @@
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="5">
-        <v>36070.183333333334</v>
+        <v>38828.729999999996</v>
       </c>
       <c r="N18" s="6">
-        <v>290</v>
+        <v>367</v>
       </c>
       <c r="O18" s="6">
-        <v>117</v>
+        <v>144</v>
       </c>
       <c r="P18" s="7">
-        <v>2.0526733788395903</v>
+        <v>2.1960359459459462</v>
       </c>
       <c r="Q18" s="8">
-        <v>10.819088888888889</v>
+        <v>11.664236805555555</v>
       </c>
       <c r="R18" s="8">
-        <v>1.8622504273504272</v>
+        <v>2.6280090277777775</v>
       </c>
       <c r="S18" s="8">
         <v>7</v>
       </c>
       <c r="T18" s="9">
-        <v>0.96581196581196582</v>
+        <v>0.92361111111111116</v>
       </c>
       <c r="U18" s="9">
-        <v>0.12820512820512819</v>
+        <v>0.125</v>
       </c>
       <c r="V18" s="9">
-        <v>0.059829059829059832</v>
+        <v>0.055555555555555552</v>
       </c>
       <c r="W18" s="9">
         <v>0</v>
@@ -4148,19 +4145,19 @@
         <v>0</v>
       </c>
       <c r="AB18" s="9">
-        <v>0.0085470085470085479</v>
+        <v>0.0069444444444444441</v>
       </c>
       <c r="AC18" s="9">
         <v>0</v>
       </c>
       <c r="AD18" s="6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AE18" s="6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AF18" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG18" s="6">
         <v>0</v>
@@ -4184,10 +4181,10 @@
         <v>0</v>
       </c>
       <c r="AN18" s="9">
-        <v>0.059829059829059832</v>
+        <v>0.0625</v>
       </c>
       <c r="AO18" s="6">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c t="s" r="AP18" s="4">
         <v>58</v>
@@ -4543,7 +4540,7 @@
         <v>19553</v>
       </c>
       <c r="B21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C21" s="4">
         <v>51</v>
@@ -4572,49 +4569,49 @@
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="5">
-        <v>52801.64166666667</v>
+        <v>59362</v>
       </c>
       <c r="N21" s="6">
-        <v>415</v>
+        <v>544</v>
       </c>
       <c r="O21" s="6">
-        <v>245</v>
+        <v>324</v>
       </c>
       <c r="P21" s="7">
-        <v>3.1500395238095238</v>
+        <v>3.3617270909090911</v>
       </c>
       <c r="Q21" s="8">
-        <v>16.72476244897959</v>
+        <v>16.952109567901235</v>
       </c>
       <c r="R21" s="8">
-        <v>6.5609049382716051</v>
+        <v>6.6585146417445493</v>
       </c>
       <c r="S21" s="8">
         <v>7</v>
       </c>
       <c r="T21" s="9">
-        <v>0.49795918367346936</v>
+        <v>0.45987654320987653</v>
       </c>
       <c r="U21" s="9">
-        <v>0.20408163265306123</v>
+        <v>0.19753086419753085</v>
       </c>
       <c r="V21" s="9">
-        <v>0.016326530612244899</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="W21" s="9">
-        <v>0.0081632653060000008</v>
+        <v>0.0092592592590000009</v>
       </c>
       <c r="X21" s="9">
-        <v>0.093877551020408165</v>
+        <v>0.07716049382716049</v>
       </c>
       <c r="Y21" s="9">
-        <v>0.0081632653061224497</v>
+        <v>0.0061728395061728392</v>
       </c>
       <c r="Z21" s="9">
-        <v>0.0040816326530612249</v>
+        <v>0.0030864197530864196</v>
       </c>
       <c r="AA21" s="9">
-        <v>0.0081632653061224497</v>
+        <v>0.012345679012345678</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
@@ -4623,19 +4620,19 @@
         <v>0</v>
       </c>
       <c r="AD21" s="6">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="AE21" s="6">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="AF21" s="6">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AG21" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH21" s="6">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AI21" s="6">
         <v>2</v>
@@ -4644,7 +4641,7 @@
         <v>1</v>
       </c>
       <c r="AK21" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL21" s="6">
         <v>0</v>
@@ -4653,10 +4650,10 @@
         <v>0</v>
       </c>
       <c r="AN21" s="9">
-        <v>0.093877551020408165</v>
+        <v>0.086419753086419748</v>
       </c>
       <c r="AO21" s="6">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c t="s" r="AP21" s="4">
         <v>58</v>
@@ -5012,7 +5009,7 @@
         <v>19565</v>
       </c>
       <c r="B24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C24" s="4">
         <v>51</v>
@@ -5043,61 +5040,61 @@
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="5">
-        <v>43031.076666666668</v>
+        <v>53742.440000000002</v>
       </c>
       <c r="N24" s="6">
-        <v>412</v>
+        <v>591</v>
       </c>
       <c r="O24" s="6">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="P24" s="7">
-        <v>3.1002412048192776</v>
+        <v>3.3049581512605042</v>
       </c>
       <c r="Q24" s="8">
-        <v>16.465551760563379</v>
+        <v>18.035351089588378</v>
       </c>
       <c r="R24" s="8">
-        <v>6.2859212121212114</v>
+        <v>7.4891579081632651</v>
       </c>
       <c r="S24" s="8">
         <v>8</v>
       </c>
       <c r="T24" s="9">
-        <v>0.426056338028169</v>
+        <v>0.36803874092009686</v>
       </c>
       <c r="U24" s="9">
-        <v>0.25</v>
+        <v>0.20289855072463769</v>
       </c>
       <c r="V24" s="9">
-        <v>0.02464788732394366</v>
+        <v>0.016908212560386472</v>
       </c>
       <c r="W24" s="9">
         <v>0</v>
       </c>
       <c r="X24" s="9">
-        <v>0.12323943661971831</v>
+        <v>0.089371980676328497</v>
       </c>
       <c r="Y24" s="9">
-        <v>0.031690140845070422</v>
+        <v>0.021739130434782608</v>
       </c>
       <c r="Z24" s="9">
         <v>0</v>
       </c>
       <c r="AA24" s="9">
-        <v>0.11619718309859155</v>
+        <v>0.089371980676328497</v>
       </c>
       <c r="AB24" s="9">
-        <v>0.052816901408450703</v>
+        <v>0.043478260869565216</v>
       </c>
       <c r="AC24" s="9">
-        <v>0</v>
+        <v>0.0096618357487922701</v>
       </c>
       <c r="AD24" s="6">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="AE24" s="6">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="AF24" s="6">
         <v>7</v>
@@ -5106,7 +5103,7 @@
         <v>0</v>
       </c>
       <c r="AH24" s="6">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AI24" s="6">
         <v>9</v>
@@ -5115,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AK24" s="6">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="AL24" s="6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AM24" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AN24" s="9">
         <v>0</v>
@@ -6111,7 +6108,7 @@
         <v>19596</v>
       </c>
       <c r="B31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C31" s="4">
         <v>51</v>
@@ -6140,70 +6137,70 @@
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="5">
-        <v>44391.561666666668</v>
+        <v>48944.869999999995</v>
       </c>
       <c r="N31" s="6">
-        <v>428</v>
+        <v>537</v>
       </c>
       <c r="O31" s="6">
-        <v>229</v>
+        <v>287</v>
       </c>
       <c r="P31" s="7">
-        <v>3.3007228915662647</v>
+        <v>3.271647509578544</v>
       </c>
       <c r="Q31" s="8">
-        <v>18.93845043859649</v>
+        <v>18.233742807017542</v>
       </c>
       <c r="R31" s="8">
-        <v>9.0296375565610862</v>
+        <v>8.3274575539568332</v>
       </c>
       <c r="S31" s="8">
         <v>7</v>
       </c>
       <c r="T31" s="9">
-        <v>0.35526315789473684</v>
+        <v>0.39649122807017545</v>
       </c>
       <c r="U31" s="9">
-        <v>0.20960698689956331</v>
+        <v>0.20905923344947736</v>
       </c>
       <c r="V31" s="9">
-        <v>0.048034934497816595</v>
+        <v>0.041811846689895474</v>
       </c>
       <c r="W31" s="9">
         <v>0</v>
       </c>
       <c r="X31" s="9">
-        <v>0.09606986899563319</v>
+        <v>0.10104529616724739</v>
       </c>
       <c r="Y31" s="9">
-        <v>0.026200873362445413</v>
+        <v>0.020905923344947737</v>
       </c>
       <c r="Z31" s="9">
         <v>0</v>
       </c>
       <c r="AA31" s="9">
-        <v>0.030567685589519649</v>
+        <v>0.024390243902439025</v>
       </c>
       <c r="AB31" s="9">
-        <v>0.056768558951965066</v>
+        <v>0.059233449477351915</v>
       </c>
       <c r="AC31" s="9">
-        <v>0.017467248908296942</v>
+        <v>0.013937282229965157</v>
       </c>
       <c r="AD31" s="6">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="AE31" s="6">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="AF31" s="6">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AG31" s="6">
         <v>0</v>
       </c>
       <c r="AH31" s="6">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="AI31" s="6">
         <v>6</v>
@@ -6215,7 +6212,7 @@
         <v>7</v>
       </c>
       <c r="AL31" s="6">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AM31" s="6">
         <v>4</v>
@@ -6733,7 +6730,7 @@
         <v>19601</v>
       </c>
       <c r="B35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C35" s="4">
         <v>51</v>
@@ -6764,61 +6761,61 @@
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="5">
-        <v>43097.611666666664</v>
+        <v>51976.509999999995</v>
       </c>
       <c r="N35" s="6">
-        <v>419</v>
+        <v>577</v>
       </c>
       <c r="O35" s="6">
-        <v>246</v>
+        <v>328</v>
       </c>
       <c r="P35" s="7">
-        <v>2.6629020304568525</v>
+        <v>3.0301459016393442</v>
       </c>
       <c r="Q35" s="8">
-        <v>16.405758943089431</v>
+        <v>17.175864024390243</v>
       </c>
       <c r="R35" s="8">
-        <v>6.0520306722689075</v>
+        <v>6.5262053459119489</v>
       </c>
       <c r="S35" s="8">
         <v>8</v>
       </c>
       <c r="T35" s="9">
-        <v>0.5</v>
+        <v>0.43292682926829268</v>
       </c>
       <c r="U35" s="9">
-        <v>0.22357723577235772</v>
+        <v>0.2347560975609756</v>
       </c>
       <c r="V35" s="9">
-        <v>0.02032520325203252</v>
+        <v>0.01524390243902439</v>
       </c>
       <c r="W35" s="9">
         <v>0</v>
       </c>
       <c r="X35" s="9">
-        <v>0.06097560975609756</v>
+        <v>0.051829268292682924</v>
       </c>
       <c r="Y35" s="9">
-        <v>0.0040650406504065045</v>
+        <v>0.0060975609756097563</v>
       </c>
       <c r="Z35" s="9">
         <v>0</v>
       </c>
       <c r="AA35" s="9">
-        <v>0.06910569105691057</v>
+        <v>0.057926829268292686</v>
       </c>
       <c r="AB35" s="9">
-        <v>0.056910569105691054</v>
+        <v>0.10365853658536585</v>
       </c>
       <c r="AC35" s="9">
-        <v>0.032520325203252036</v>
+        <v>0.024390243902439025</v>
       </c>
       <c r="AD35" s="6">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="AE35" s="6">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="AF35" s="6">
         <v>5</v>
@@ -6827,19 +6824,19 @@
         <v>0</v>
       </c>
       <c r="AH35" s="6">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AI35" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ35" s="6">
         <v>0</v>
       </c>
       <c r="AK35" s="6">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="AL35" s="6">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="AM35" s="6">
         <v>8</v>
@@ -7181,7 +7178,7 @@
         <v>422</v>
       </c>
       <c r="O38" s="6">
-        <v>66</v>
+        <v>247</v>
       </c>
       <c r="P38" s="7">
         <v>3.7685453237410074</v>
@@ -7199,16 +7196,16 @@
         <v>0.63157894736842102</v>
       </c>
       <c r="U38" s="9">
-        <v>0.030303030303030304</v>
+        <v>0.032388663967611336</v>
       </c>
       <c r="V38" s="9">
-        <v>0.015151515151515152</v>
+        <v>0.0080971659919028341</v>
       </c>
       <c r="W38" s="9">
         <v>0</v>
       </c>
       <c r="X38" s="9">
-        <v>0.015151515151515152</v>
+        <v>0.012145748987854251</v>
       </c>
       <c r="Y38" s="9">
         <v>0</v>
@@ -7217,43 +7214,43 @@
         <v>0</v>
       </c>
       <c r="AA38" s="9">
-        <v>0</v>
+        <v>0.004048582995951417</v>
       </c>
       <c r="AB38" s="9">
         <v>0</v>
       </c>
       <c r="AC38" s="9">
-        <v>0</v>
+        <v>0.0080971659919028341</v>
       </c>
       <c r="AD38" s="6">
+        <v>8</v>
+      </c>
+      <c r="AE38" s="6">
+        <v>8</v>
+      </c>
+      <c r="AF38" s="6">
         <v>2</v>
       </c>
-      <c r="AE38" s="6">
+      <c r="AG38" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH38" s="6">
+        <v>3</v>
+      </c>
+      <c r="AI38" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ38" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK38" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL38" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM38" s="6">
         <v>2</v>
-      </c>
-      <c r="AF38" s="6">
-        <v>1</v>
-      </c>
-      <c r="AG38" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH38" s="6">
-        <v>1</v>
-      </c>
-      <c r="AI38" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ38" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK38" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL38" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM38" s="6">
-        <v>0</v>
       </c>
       <c r="AN38" s="9">
         <v>0</v>
@@ -7458,7 +7455,7 @@
         <v>19615</v>
       </c>
       <c r="B40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C40" s="4">
         <v>51</v>
@@ -7489,70 +7486,70 @@
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="5">
-        <v>41471.33666666667</v>
+        <v>45697.510000000002</v>
       </c>
       <c r="N40" s="6">
-        <v>420</v>
+        <v>551</v>
       </c>
       <c r="O40" s="6">
-        <v>333</v>
+        <v>446</v>
       </c>
       <c r="P40" s="7">
-        <v>2.8418979166666669</v>
+        <v>2.9595780316344467</v>
       </c>
       <c r="Q40" s="8">
-        <v>19.208536585365852</v>
+        <v>22.123787528868363</v>
       </c>
       <c r="R40" s="8">
-        <v>10.135905787781351</v>
+        <v>12.909495192307693</v>
       </c>
       <c r="S40" s="8">
         <v>7</v>
       </c>
       <c r="T40" s="9">
-        <v>0.34756097560975607</v>
+        <v>0.28406466512702078</v>
       </c>
       <c r="U40" s="9">
-        <v>0.23123123123123124</v>
+        <v>0.23542600896860988</v>
       </c>
       <c r="V40" s="9">
-        <v>0.012012012012012012</v>
+        <v>0.011210762331838564</v>
       </c>
       <c r="W40" s="9">
         <v>0</v>
       </c>
       <c r="X40" s="9">
-        <v>0.1111111111111111</v>
+        <v>0.09641255605381166</v>
       </c>
       <c r="Y40" s="9">
-        <v>0.0090090090090090089</v>
+        <v>0.0067264573991031393</v>
       </c>
       <c r="Z40" s="9">
         <v>0</v>
       </c>
       <c r="AA40" s="9">
-        <v>0.06006006006006006</v>
+        <v>0.049327354260089683</v>
       </c>
       <c r="AB40" s="9">
-        <v>0.0090090090090090089</v>
+        <v>0.0067264573991031393</v>
       </c>
       <c r="AC40" s="9">
-        <v>0.066066066066066062</v>
+        <v>0.091928251121076235</v>
       </c>
       <c r="AD40" s="6">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="AE40" s="6">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="AF40" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG40" s="6">
         <v>0</v>
       </c>
       <c r="AH40" s="6">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="AI40" s="6">
         <v>3</v>
@@ -7561,13 +7558,13 @@
         <v>0</v>
       </c>
       <c r="AK40" s="6">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AL40" s="6">
         <v>3</v>
       </c>
       <c r="AM40" s="6">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="AN40" s="9">
         <v>0</v>
@@ -7650,7 +7647,7 @@
         <v>668</v>
       </c>
       <c r="O41" s="6">
-        <v>319</v>
+        <v>402</v>
       </c>
       <c r="P41" s="7">
         <v>9.9941057926829266</v>
@@ -7668,64 +7665,64 @@
         <v>0.30597014925373134</v>
       </c>
       <c r="U41" s="9">
-        <v>0.13479623824451412</v>
+        <v>0.14676616915422885</v>
       </c>
       <c r="V41" s="9">
-        <v>0.003134796238244514</v>
+        <v>0.0049751243781094526</v>
       </c>
       <c r="W41" s="9">
         <v>0</v>
       </c>
       <c r="X41" s="9">
-        <v>0.028213166144200628</v>
+        <v>0.02736318407960199</v>
       </c>
       <c r="Y41" s="9">
-        <v>0</v>
+        <v>0.0024875621890547263</v>
       </c>
       <c r="Z41" s="9">
-        <v>0.003134796238244514</v>
+        <v>0.0024875621890547263</v>
       </c>
       <c r="AA41" s="9">
-        <v>0.072100313479623826</v>
+        <v>0.092039800995024873</v>
       </c>
       <c r="AB41" s="9">
-        <v>0.025078369905956112</v>
+        <v>0.022388059701492536</v>
       </c>
       <c r="AC41" s="9">
-        <v>0.006269592476489028</v>
+        <v>0.0049751243781094526</v>
       </c>
       <c r="AD41" s="6">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="AE41" s="6">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="AF41" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG41" s="6">
         <v>0</v>
       </c>
       <c r="AH41" s="6">
+        <v>11</v>
+      </c>
+      <c r="AI41" s="6">
+        <v>1</v>
+      </c>
+      <c r="AJ41" s="6">
+        <v>1</v>
+      </c>
+      <c r="AK41" s="6">
+        <v>37</v>
+      </c>
+      <c r="AL41" s="6">
         <v>9</v>
-      </c>
-      <c r="AI41" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ41" s="6">
-        <v>1</v>
-      </c>
-      <c r="AK41" s="6">
-        <v>23</v>
-      </c>
-      <c r="AL41" s="6">
-        <v>8</v>
       </c>
       <c r="AM41" s="6">
         <v>2</v>
       </c>
       <c r="AN41" s="9">
-        <v>0.0094043887147335428</v>
+        <v>0.007462686567164179</v>
       </c>
       <c r="AO41" s="6">
         <v>3</v>
@@ -8340,7 +8337,7 @@
         <v>19624</v>
       </c>
       <c r="B46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C46" s="4">
         <v>51</v>
@@ -8369,70 +8366,70 @@
       </c>
       <c r="L46" s="4"/>
       <c r="M46" s="5">
-        <v>23033.359999999997</v>
+        <v>28066.539999999997</v>
       </c>
       <c r="N46" s="6">
-        <v>237</v>
+        <v>331</v>
       </c>
       <c r="O46" s="6">
-        <v>110</v>
+        <v>157</v>
       </c>
       <c r="P46" s="7">
-        <v>2.5236170212765954</v>
+        <v>2.6206948640483385</v>
       </c>
       <c r="Q46" s="8">
-        <v>13.954091818181819</v>
+        <v>14.670807643312102</v>
       </c>
       <c r="R46" s="8">
-        <v>5.3781660000000002</v>
+        <v>5.8083328767123295</v>
       </c>
       <c r="S46" s="8">
         <v>7</v>
       </c>
       <c r="T46" s="9">
-        <v>0.67272727272727273</v>
+        <v>0.61146496815286622</v>
       </c>
       <c r="U46" s="9">
-        <v>0.25454545454545452</v>
+        <v>0.20382165605095542</v>
       </c>
       <c r="V46" s="9">
-        <v>0.018181818181818181</v>
+        <v>0.019108280254777069</v>
       </c>
       <c r="W46" s="9">
-        <v>0.00909090909</v>
+        <v>0.0063694267510000001</v>
       </c>
       <c r="X46" s="9">
-        <v>0.10000000000000001</v>
+        <v>0.082802547770700632</v>
       </c>
       <c r="Y46" s="9">
-        <v>0.054545454545454543</v>
+        <v>0.038216560509554139</v>
       </c>
       <c r="Z46" s="9">
-        <v>0.0090909090909090905</v>
+        <v>0.006369426751592357</v>
       </c>
       <c r="AA46" s="9">
-        <v>0.14545454545454545</v>
+        <v>0.10828025477707007</v>
       </c>
       <c r="AB46" s="9">
-        <v>0.018181818181818181</v>
+        <v>0.012738853503184714</v>
       </c>
       <c r="AC46" s="9">
-        <v>0.018181818181818181</v>
+        <v>0.012738853503184714</v>
       </c>
       <c r="AD46" s="6">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="AE46" s="6">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="AF46" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG46" s="6">
         <v>1</v>
       </c>
       <c r="AH46" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AI46" s="6">
         <v>6</v>
@@ -8441,7 +8438,7 @@
         <v>1</v>
       </c>
       <c r="AK46" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AL46" s="6">
         <v>2</v>
@@ -9375,7 +9372,7 @@
         <v>19647</v>
       </c>
       <c r="B53" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C53" s="4">
         <v>51</v>
@@ -9404,40 +9401,40 @@
       </c>
       <c r="L53" s="4"/>
       <c r="M53" s="5">
-        <v>29951.460000000003</v>
+        <v>33502.190000000002</v>
       </c>
       <c r="N53" s="6">
-        <v>268</v>
+        <v>350</v>
       </c>
       <c r="O53" s="6">
-        <v>190</v>
+        <v>238</v>
       </c>
       <c r="P53" s="7">
-        <v>4.6347377289377292</v>
+        <v>6.7962293296089387</v>
       </c>
       <c r="Q53" s="8">
-        <v>21.511403157894737</v>
+        <v>24.087534873949579</v>
       </c>
       <c r="R53" s="8">
-        <v>8.8296494736842099</v>
+        <v>9.9695382352941184</v>
       </c>
       <c r="S53" s="8">
         <v>8</v>
       </c>
       <c r="T53" s="9">
-        <v>0.27368421052631581</v>
+        <v>0.22268907563025211</v>
       </c>
       <c r="U53" s="9">
-        <v>0.073684210526315783</v>
+        <v>0.067226890756302518</v>
       </c>
       <c r="V53" s="9">
-        <v>0</v>
+        <v>0.0042016806722689074</v>
       </c>
       <c r="W53" s="9">
-        <v>0.005263157894</v>
+        <v>0.0042016806720000001</v>
       </c>
       <c r="X53" s="9">
-        <v>0.042105263157894736</v>
+        <v>0.033613445378151259</v>
       </c>
       <c r="Y53" s="9">
         <v>0</v>
@@ -9446,22 +9443,22 @@
         <v>0</v>
       </c>
       <c r="AA53" s="9">
-        <v>0.005263157894736842</v>
+        <v>0.0084033613445378148</v>
       </c>
       <c r="AB53" s="9">
-        <v>0.026315789473684209</v>
+        <v>0.02100840336134454</v>
       </c>
       <c r="AC53" s="9">
         <v>0</v>
       </c>
       <c r="AD53" s="6">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AE53" s="6">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AF53" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG53" s="6">
         <v>1</v>
@@ -9476,7 +9473,7 @@
         <v>0</v>
       </c>
       <c r="AK53" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL53" s="6">
         <v>5</v>
@@ -9530,7 +9527,7 @@
         <v>19648</v>
       </c>
       <c r="B54" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C54" s="4">
         <v>51</v>
@@ -9561,79 +9558,79 @@
       </c>
       <c r="L54" s="4"/>
       <c r="M54" s="5">
-        <v>33276.949999999997</v>
+        <v>38383.399999999987</v>
       </c>
       <c r="N54" s="6">
-        <v>324</v>
+        <v>429</v>
       </c>
       <c r="O54" s="6">
-        <v>178</v>
+        <v>241</v>
       </c>
       <c r="P54" s="7">
-        <v>6.2680731249999999</v>
+        <v>5.9278040000000001</v>
       </c>
       <c r="Q54" s="8">
-        <v>19.673969662921351</v>
+        <v>21.347441078838173</v>
       </c>
       <c r="R54" s="8">
-        <v>6.2542387283237</v>
+        <v>8.2714893617021268</v>
       </c>
       <c r="S54" s="8">
         <v>7</v>
       </c>
       <c r="T54" s="9">
-        <v>0.33146067415730335</v>
+        <v>0.29045643153526973</v>
       </c>
       <c r="U54" s="9">
-        <v>0.12921348314606743</v>
+        <v>0.12448132780082988</v>
       </c>
       <c r="V54" s="9">
-        <v>0.033707865168539325</v>
+        <v>0.037344398340248962</v>
       </c>
       <c r="W54" s="9">
         <v>0</v>
       </c>
       <c r="X54" s="9">
-        <v>0.056179775280898875</v>
+        <v>0.062240663900414939</v>
       </c>
       <c r="Y54" s="9">
-        <v>0.011235955056179775</v>
+        <v>0.012448132780082987</v>
       </c>
       <c r="Z54" s="9">
         <v>0</v>
       </c>
       <c r="AA54" s="9">
-        <v>0.0449438202247191</v>
+        <v>0.037344398340248962</v>
       </c>
       <c r="AB54" s="9">
-        <v>0.02247191011235955</v>
+        <v>0.016597510373443983</v>
       </c>
       <c r="AC54" s="9">
         <v>0</v>
       </c>
       <c r="AD54" s="6">
+        <v>40</v>
+      </c>
+      <c r="AE54" s="6">
         <v>30</v>
       </c>
-      <c r="AE54" s="6">
-        <v>23</v>
-      </c>
       <c r="AF54" s="6">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AG54" s="6">
         <v>0</v>
       </c>
       <c r="AH54" s="6">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AI54" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ54" s="6">
         <v>0</v>
       </c>
       <c r="AK54" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL54" s="6">
         <v>4</v>
@@ -9687,7 +9684,7 @@
         <v>19649</v>
       </c>
       <c r="B55" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C55" s="4">
         <v>51</v>
@@ -9716,82 +9713,82 @@
       </c>
       <c r="L55" s="4"/>
       <c r="M55" s="5">
-        <v>48284.459999999999</v>
+        <v>55698.099999999999</v>
       </c>
       <c r="N55" s="6">
-        <v>458</v>
+        <v>624</v>
       </c>
       <c r="O55" s="6">
-        <v>187</v>
+        <v>260</v>
       </c>
       <c r="P55" s="7">
-        <v>2.2450452702702703</v>
+        <v>3.2038294214876033</v>
       </c>
       <c r="Q55" s="8">
-        <v>17.078877005347593</v>
+        <v>17.771153846153847</v>
       </c>
       <c r="R55" s="8">
-        <v>7.2728364640883978</v>
+        <v>7.2039844621513947</v>
       </c>
       <c r="S55" s="8">
         <v>8</v>
       </c>
       <c r="T55" s="9">
-        <v>0.47593582887700536</v>
+        <v>0.44615384615384618</v>
       </c>
       <c r="U55" s="9">
-        <v>0.32085561497326204</v>
+        <v>0.27692307692307694</v>
       </c>
       <c r="V55" s="9">
-        <v>0.021390374331550801</v>
+        <v>0.023076923076923078</v>
       </c>
       <c r="W55" s="9">
-        <v>0.010695187165</v>
+        <v>0.0076923076919999996</v>
       </c>
       <c r="X55" s="9">
-        <v>0.23529411764705882</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="Y55" s="9">
-        <v>0.021390374331550801</v>
+        <v>0.023076923076923078</v>
       </c>
       <c r="Z55" s="9">
         <v>0</v>
       </c>
       <c r="AA55" s="9">
-        <v>0.058823529411764705</v>
+        <v>0.057692307692307696</v>
       </c>
       <c r="AB55" s="9">
-        <v>0.048128342245989303</v>
+        <v>0.038461538461538464</v>
       </c>
       <c r="AC55" s="9">
         <v>0</v>
       </c>
       <c r="AD55" s="6">
+        <v>89</v>
+      </c>
+      <c r="AE55" s="6">
         <v>72</v>
       </c>
-      <c r="AE55" s="6">
-        <v>60</v>
-      </c>
       <c r="AF55" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AG55" s="6">
         <v>2</v>
       </c>
       <c r="AH55" s="6">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AI55" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AJ55" s="6">
         <v>0</v>
       </c>
       <c r="AK55" s="6">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AL55" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AM55" s="6">
         <v>0</v>
@@ -9997,7 +9994,7 @@
         <v>19654</v>
       </c>
       <c r="B57" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="s" r="C57" s="4">
         <v>51</v>
@@ -10026,82 +10023,82 @@
       </c>
       <c r="L57" s="4"/>
       <c r="M57" s="5">
-        <v>29293.781999999996</v>
+        <v>38354.859999999993</v>
       </c>
       <c r="N57" s="6">
-        <v>252</v>
+        <v>462</v>
       </c>
       <c r="O57" s="6">
-        <v>108</v>
+        <v>210</v>
       </c>
       <c r="P57" s="7">
-        <v>3.5140004</v>
+        <v>3.6241687361419066</v>
       </c>
       <c r="Q57" s="8">
-        <v>15.308795370370369</v>
+        <v>16.126983809523811</v>
       </c>
       <c r="R57" s="8">
-        <v>5.2138895833333327</v>
+        <v>5.4694876923076921</v>
       </c>
       <c r="S57" s="8">
         <v>8</v>
       </c>
       <c r="T57" s="9">
-        <v>0.53703703703703709</v>
+        <v>0.48095238095238096</v>
       </c>
       <c r="U57" s="9">
-        <v>0.27777777777777779</v>
+        <v>0.20952380952380953</v>
       </c>
       <c r="V57" s="9">
-        <v>0.018518518518518517</v>
+        <v>0.014285714285714285</v>
       </c>
       <c r="W57" s="9">
         <v>0</v>
       </c>
       <c r="X57" s="9">
-        <v>0.15740740740740741</v>
+        <v>0.10476190476190476</v>
       </c>
       <c r="Y57" s="9">
-        <v>0.07407407407407407</v>
+        <v>0.047619047619047616</v>
       </c>
       <c r="Z57" s="9">
         <v>0</v>
       </c>
       <c r="AA57" s="9">
-        <v>0.1388888888888889</v>
+        <v>0.10952380952380952</v>
       </c>
       <c r="AB57" s="9">
-        <v>0.064814814814814811</v>
+        <v>0.047619047619047616</v>
       </c>
       <c r="AC57" s="9">
         <v>0</v>
       </c>
       <c r="AD57" s="6">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="AE57" s="6">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="AF57" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG57" s="6">
         <v>0</v>
       </c>
       <c r="AH57" s="6">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AI57" s="6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AJ57" s="6">
         <v>0</v>
       </c>
       <c r="AK57" s="6">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AL57" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AM57" s="6">
         <v>0</v>
@@ -10249,7 +10246,7 @@
         <v>19657</v>
       </c>
       <c r="B59" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C59" s="4">
         <v>51</v>
@@ -10280,82 +10277,82 @@
       </c>
       <c r="L59" s="4"/>
       <c r="M59" s="5">
-        <v>34192.981666666667</v>
+        <v>37571.270000000004</v>
       </c>
       <c r="N59" s="6">
-        <v>306</v>
+        <v>390</v>
       </c>
       <c r="O59" s="6">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="P59" s="7">
-        <v>5.791216216216216</v>
+        <v>6.1220316622691291</v>
       </c>
       <c r="Q59" s="8">
-        <v>18.452992307692309</v>
+        <v>19.215686764705882</v>
       </c>
       <c r="R59" s="8">
-        <v>5.8300006451612898</v>
+        <v>6.2451326732673271</v>
       </c>
       <c r="S59" s="8">
         <v>7</v>
       </c>
       <c r="T59" s="9">
-        <v>0.23076923076923078</v>
+        <v>0.19607843137254902</v>
       </c>
       <c r="U59" s="9">
-        <v>0.24203821656050956</v>
+        <v>0.23414634146341465</v>
       </c>
       <c r="V59" s="9">
-        <v>0.031847133757961783</v>
+        <v>0.024390243902439025</v>
       </c>
       <c r="W59" s="9">
-        <v>0</v>
+        <v>0.0048780487799999998</v>
       </c>
       <c r="X59" s="9">
-        <v>0.019108280254777069</v>
+        <v>0.014634146341463415</v>
       </c>
       <c r="Y59" s="9">
-        <v>0</v>
+        <v>0.0048780487804878049</v>
       </c>
       <c r="Z59" s="9">
-        <v>0.006369426751592357</v>
+        <v>0.0097560975609756097</v>
       </c>
       <c r="AA59" s="9">
-        <v>0.006369426751592357</v>
+        <v>0.0097560975609756097</v>
       </c>
       <c r="AB59" s="9">
-        <v>0.16560509554140126</v>
+        <v>0.16585365853658537</v>
       </c>
       <c r="AC59" s="9">
-        <v>0.038216560509554139</v>
+        <v>0.029268292682926831</v>
       </c>
       <c r="AD59" s="6">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="AE59" s="6">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="AF59" s="6">
         <v>5</v>
       </c>
       <c r="AG59" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH59" s="6">
         <v>3</v>
       </c>
       <c r="AI59" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ59" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AK59" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL59" s="6">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="AM59" s="6">
         <v>6</v>
@@ -10620,7 +10617,7 @@
         <v>0.0052493438320209973</v>
       </c>
       <c r="W61" s="9">
-        <v>0</v>
+        <v>0.0026246719160000001</v>
       </c>
       <c r="X61" s="9">
         <v>0.020997375328083989</v>
@@ -10650,7 +10647,7 @@
         <v>2</v>
       </c>
       <c r="AG61" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH61" s="6">
         <v>8</v>
@@ -11441,7 +11438,7 @@
         <v>19685</v>
       </c>
       <c r="B67" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C67" s="4">
         <v>51</v>
@@ -11472,64 +11469,64 @@
       </c>
       <c r="L67" s="4"/>
       <c r="M67" s="5">
-        <v>25134.246666666662</v>
+        <v>26353.790000000001</v>
       </c>
       <c r="N67" s="6">
-        <v>241</v>
+        <v>292</v>
       </c>
       <c r="O67" s="6">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="P67" s="7">
-        <v>7.1342138211382107</v>
+        <v>7.3023645270270263</v>
       </c>
       <c r="Q67" s="8">
-        <v>19.864349197860964</v>
+        <v>22.114495813953489</v>
       </c>
       <c r="R67" s="8">
-        <v>7.545269032258064</v>
+        <v>10.00288659217877</v>
       </c>
       <c r="S67" s="8">
         <v>7</v>
       </c>
       <c r="T67" s="9">
-        <v>0.30481283422459893</v>
+        <v>0.27906976744186046</v>
       </c>
       <c r="U67" s="9">
-        <v>0.28723404255319152</v>
+        <v>0.31018518518518517</v>
       </c>
       <c r="V67" s="9">
-        <v>0.0053191489361702126</v>
+        <v>0.0092592592592592587</v>
       </c>
       <c r="W67" s="9">
         <v>0</v>
       </c>
       <c r="X67" s="9">
-        <v>0.026595744680851064</v>
+        <v>0.023148148148148147</v>
       </c>
       <c r="Y67" s="9">
-        <v>0.0053191489361702126</v>
+        <v>0.0046296296296296294</v>
       </c>
       <c r="Z67" s="9">
-        <v>0.0053191489361702126</v>
+        <v>0.0046296296296296294</v>
       </c>
       <c r="AA67" s="9">
-        <v>0.25531914893617019</v>
+        <v>0.24537037037037038</v>
       </c>
       <c r="AB67" s="9">
         <v>0</v>
       </c>
       <c r="AC67" s="9">
-        <v>0</v>
+        <v>0.046296296296296294</v>
       </c>
       <c r="AD67" s="6">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="AE67" s="6">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="AF67" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG67" s="6">
         <v>0</v>
@@ -11544,13 +11541,13 @@
         <v>1</v>
       </c>
       <c r="AK67" s="6">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="AL67" s="6">
         <v>0</v>
       </c>
       <c r="AM67" s="6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AN67" s="9">
         <v>0</v>
@@ -11598,7 +11595,7 @@
         <v>19687</v>
       </c>
       <c r="B68" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C68" s="4">
         <v>51</v>
@@ -11629,40 +11626,40 @@
       </c>
       <c r="L68" s="4"/>
       <c r="M68" s="5">
-        <v>34525.411666666667</v>
+        <v>34514.839999999997</v>
       </c>
       <c r="N68" s="6">
-        <v>379</v>
+        <v>446</v>
       </c>
       <c r="O68" s="6">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P68" s="7">
-        <v>6.1386885885885887</v>
+        <v>6.1113966580976857</v>
       </c>
       <c r="Q68" s="8">
-        <v>22.46709487179487</v>
+        <v>20.849668000000001</v>
       </c>
       <c r="R68" s="8">
-        <v>11.38225806451613</v>
+        <v>10.090171794871795</v>
       </c>
       <c r="S68" s="8">
         <v>7</v>
       </c>
       <c r="T68" s="9">
-        <v>0.38461538461538464</v>
+        <v>0.41999999999999998</v>
       </c>
       <c r="U68" s="9">
-        <v>0.38461538461538464</v>
+        <v>0.44</v>
       </c>
       <c r="V68" s="9">
-        <v>0.076923076923076927</v>
+        <v>0.10000000000000001</v>
       </c>
       <c r="W68" s="9">
         <v>0</v>
       </c>
       <c r="X68" s="9">
-        <v>0.05128205128205128</v>
+        <v>0.059999999999999998</v>
       </c>
       <c r="Y68" s="9">
         <v>0</v>
@@ -11671,40 +11668,40 @@
         <v>0</v>
       </c>
       <c r="AA68" s="9">
-        <v>0.33333333333333331</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="AB68" s="9">
-        <v>0</v>
+        <v>0.040000000000000001</v>
       </c>
       <c r="AC68" s="9">
         <v>0</v>
       </c>
       <c r="AD68" s="6">
+        <v>28</v>
+      </c>
+      <c r="AE68" s="6">
+        <v>22</v>
+      </c>
+      <c r="AF68" s="6">
+        <v>5</v>
+      </c>
+      <c r="AG68" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH68" s="6">
+        <v>3</v>
+      </c>
+      <c r="AI68" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ68" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK68" s="6">
         <v>18</v>
       </c>
-      <c r="AE68" s="6">
-        <v>15</v>
-      </c>
-      <c r="AF68" s="6">
-        <v>3</v>
-      </c>
-      <c r="AG68" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH68" s="6">
+      <c r="AL68" s="6">
         <v>2</v>
-      </c>
-      <c r="AI68" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ68" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK68" s="6">
-        <v>13</v>
-      </c>
-      <c r="AL68" s="6">
-        <v>0</v>
       </c>
       <c r="AM68" s="6">
         <v>0</v>
@@ -11912,7 +11909,7 @@
         <v>19689</v>
       </c>
       <c r="B70" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C70" s="4">
         <v>51</v>
@@ -11943,61 +11940,61 @@
       </c>
       <c r="L70" s="4"/>
       <c r="M70" s="5">
-        <v>38406.748333333329</v>
+        <v>44123.419999999998</v>
       </c>
       <c r="N70" s="6">
-        <v>309</v>
+        <v>416</v>
       </c>
       <c r="O70" s="6">
-        <v>166</v>
+        <v>222</v>
       </c>
       <c r="P70" s="7">
-        <v>3.260664308681672</v>
+        <v>3.4512329355608595</v>
       </c>
       <c r="Q70" s="8">
-        <v>10.685039759036144</v>
+        <v>11.006155855855855</v>
       </c>
       <c r="R70" s="8">
-        <v>2.8380715686274507</v>
+        <v>2.9029338028169014</v>
       </c>
       <c r="S70" s="8">
         <v>7</v>
       </c>
       <c r="T70" s="9">
-        <v>0.83734939759036142</v>
+        <v>0.82432432432432434</v>
       </c>
       <c r="U70" s="9">
-        <v>0.5</v>
+        <v>0.49099099099099097</v>
       </c>
       <c r="V70" s="9">
-        <v>0.006024096385542169</v>
+        <v>0.0045045045045045045</v>
       </c>
       <c r="W70" s="9">
         <v>0</v>
       </c>
       <c r="X70" s="9">
-        <v>0.054216867469879519</v>
+        <v>0.054054054054054057</v>
       </c>
       <c r="Y70" s="9">
-        <v>0.12650602409638553</v>
+        <v>0.11261261261261261</v>
       </c>
       <c r="Z70" s="9">
         <v>0</v>
       </c>
       <c r="AA70" s="9">
-        <v>0.44578313253012047</v>
+        <v>0.44144144144144143</v>
       </c>
       <c r="AB70" s="9">
-        <v>0.066265060240963861</v>
+        <v>0.04954954954954955</v>
       </c>
       <c r="AC70" s="9">
         <v>0</v>
       </c>
       <c r="AD70" s="6">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="AE70" s="6">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="AF70" s="6">
         <v>1</v>
@@ -12006,16 +12003,16 @@
         <v>0</v>
       </c>
       <c r="AH70" s="6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AI70" s="6">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="AJ70" s="6">
         <v>0</v>
       </c>
       <c r="AK70" s="6">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="AL70" s="6">
         <v>11</v>
@@ -12379,7 +12376,7 @@
         <v>19694</v>
       </c>
       <c r="B73" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C73" s="4">
         <v>51</v>
@@ -12410,85 +12407,85 @@
       </c>
       <c r="L73" s="4"/>
       <c r="M73" s="5">
-        <v>49140.186666666668</v>
+        <v>49657.710000000006</v>
       </c>
       <c r="N73" s="6">
-        <v>419</v>
+        <v>499</v>
       </c>
       <c r="O73" s="6">
-        <v>292</v>
+        <v>346</v>
       </c>
       <c r="P73" s="7">
-        <v>7.1830949880668262</v>
+        <v>6.6024818913480887</v>
       </c>
       <c r="Q73" s="8">
-        <v>29.598230479452056</v>
+        <v>29.708670520231216</v>
       </c>
       <c r="R73" s="8">
-        <v>15.531436896551723</v>
+        <v>16.204699709302325</v>
       </c>
       <c r="S73" s="8">
         <v>7</v>
       </c>
       <c r="T73" s="9">
-        <v>0.11986301369863013</v>
+        <v>0.10982658959537572</v>
       </c>
       <c r="U73" s="9">
-        <v>0.2226027397260274</v>
+        <v>0.21965317919075145</v>
       </c>
       <c r="V73" s="9">
-        <v>0.071917808219178078</v>
+        <v>0.06358381502890173</v>
       </c>
       <c r="W73" s="9">
-        <v>0.0034246575339999998</v>
+        <v>0.0028901734099999999</v>
       </c>
       <c r="X73" s="9">
-        <v>0.041095890410958902</v>
+        <v>0.049132947976878616</v>
       </c>
       <c r="Y73" s="9">
-        <v>0.0034246575342465752</v>
+        <v>0.0028901734104046241</v>
       </c>
       <c r="Z73" s="9">
-        <v>0</v>
+        <v>0.0028901734104046241</v>
       </c>
       <c r="AA73" s="9">
-        <v>0.013698630136986301</v>
+        <v>0.011560693641618497</v>
       </c>
       <c r="AB73" s="9">
-        <v>0.017123287671232876</v>
+        <v>0.017341040462427744</v>
       </c>
       <c r="AC73" s="9">
-        <v>0.095890410958904104</v>
+        <v>0.089595375722543349</v>
       </c>
       <c r="AD73" s="6">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="AE73" s="6">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="AF73" s="6">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AG73" s="6">
         <v>1</v>
       </c>
       <c r="AH73" s="6">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="AI73" s="6">
         <v>1</v>
       </c>
       <c r="AJ73" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK73" s="6">
         <v>4</v>
       </c>
       <c r="AL73" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AM73" s="6">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AN73" s="9">
         <v>0</v>
@@ -14926,7 +14923,7 @@
         <v>19730</v>
       </c>
       <c r="B90" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C90" s="4">
         <v>51</v>
@@ -14955,67 +14952,67 @@
       </c>
       <c r="L90" s="4"/>
       <c r="M90" s="5">
-        <v>57734.903333333328</v>
+        <v>62360.949999999997</v>
       </c>
       <c r="N90" s="6">
-        <v>502</v>
+        <v>640</v>
       </c>
       <c r="O90" s="6">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="P90" s="7">
-        <v>6.4565013861386138</v>
+        <v>6.1405795031055899</v>
       </c>
       <c r="Q90" s="8">
-        <v>22.940111333333334</v>
+        <v>23.887213756613757</v>
       </c>
       <c r="R90" s="8">
-        <v>8.9715879194630865</v>
+        <v>10.114715957446808</v>
       </c>
       <c r="S90" s="8">
         <v>8</v>
       </c>
       <c r="T90" s="9">
-        <v>0.13333333333333333</v>
+        <v>0.12169312169312169</v>
       </c>
       <c r="U90" s="9">
-        <v>0.26666666666666666</v>
+        <v>0.26455026455026454</v>
       </c>
       <c r="V90" s="9">
-        <v>0.02</v>
+        <v>0.021164021164021163</v>
       </c>
       <c r="W90" s="9">
-        <v>0</v>
+        <v>0.0052910052909999998</v>
       </c>
       <c r="X90" s="9">
-        <v>0.013333333333333334</v>
+        <v>0.010582010582010581</v>
       </c>
       <c r="Y90" s="9">
         <v>0</v>
       </c>
       <c r="Z90" s="9">
-        <v>0</v>
+        <v>0.0052910052910052907</v>
       </c>
       <c r="AA90" s="9">
-        <v>0.013333333333333334</v>
+        <v>0.010582010582010581</v>
       </c>
       <c r="AB90" s="9">
-        <v>0.040000000000000001</v>
+        <v>0.042328042328042326</v>
       </c>
       <c r="AC90" s="9">
-        <v>0.16</v>
+        <v>0.15873015873015872</v>
       </c>
       <c r="AD90" s="6">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="AE90" s="6">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="AF90" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG90" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH90" s="6">
         <v>2</v>
@@ -15024,22 +15021,22 @@
         <v>0</v>
       </c>
       <c r="AJ90" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK90" s="6">
         <v>2</v>
       </c>
       <c r="AL90" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AM90" s="6">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="AN90" s="9">
-        <v>0.026666666666666668</v>
+        <v>0.026455026455026454</v>
       </c>
       <c r="AO90" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c t="s" r="AP90" s="4">
         <v>58</v>
@@ -16430,7 +16427,7 @@
         <v>19749</v>
       </c>
       <c r="B100" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C100" s="4">
         <v>51</v>
@@ -16459,49 +16456,49 @@
       </c>
       <c r="L100" s="4"/>
       <c r="M100" s="5">
-        <v>30329.565000000002</v>
+        <v>31718.230000000003</v>
       </c>
       <c r="N100" s="6">
-        <v>277</v>
+        <v>342</v>
       </c>
       <c r="O100" s="6">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="P100" s="7">
-        <v>9.1926340823970047</v>
+        <v>9.1982722560975603</v>
       </c>
       <c r="Q100" s="8">
-        <v>29.167873026315789</v>
+        <v>30.045637172774867</v>
       </c>
       <c r="R100" s="8">
-        <v>11.915667333333333</v>
+        <v>12.947884126984126</v>
       </c>
       <c r="S100" s="8">
         <v>8</v>
       </c>
       <c r="T100" s="9">
-        <v>0.10526315789473684</v>
+        <v>0.083769633507853408</v>
       </c>
       <c r="U100" s="9">
-        <v>0.10526315789473684</v>
+        <v>0.09947643979057591</v>
       </c>
       <c r="V100" s="9">
-        <v>0.078947368421052627</v>
+        <v>0.078534031413612565</v>
       </c>
       <c r="W100" s="9">
-        <v>0.0065789473680000002</v>
+        <v>0.0052356020940000003</v>
       </c>
       <c r="X100" s="9">
-        <v>0.039473684210526314</v>
+        <v>0.031413612565445025</v>
       </c>
       <c r="Y100" s="9">
-        <v>0.013157894736842105</v>
+        <v>0.010471204188481676</v>
       </c>
       <c r="Z100" s="9">
-        <v>0.0065789473684210523</v>
+        <v>0.005235602094240838</v>
       </c>
       <c r="AA100" s="9">
-        <v>0.013157894736842105</v>
+        <v>0.010471204188481676</v>
       </c>
       <c r="AB100" s="9">
         <v>0</v>
@@ -16510,13 +16507,13 @@
         <v>0</v>
       </c>
       <c r="AD100" s="6">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="AE100" s="6">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="AF100" s="6">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="AG100" s="6">
         <v>1</v>
@@ -16585,7 +16582,7 @@
         <v>19752</v>
       </c>
       <c r="B101" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C101" s="4">
         <v>51</v>
@@ -16614,64 +16611,64 @@
       </c>
       <c r="L101" s="4"/>
       <c r="M101" s="5">
-        <v>25637.394999999993</v>
+        <v>27214.859999999997</v>
       </c>
       <c r="N101" s="6">
-        <v>243</v>
+        <v>301</v>
       </c>
       <c r="O101" s="6">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="P101" s="7">
-        <v>6.1071224066390037</v>
+        <v>6.7369558528428088</v>
       </c>
       <c r="Q101" s="8">
-        <v>22.256134027777776</v>
+        <v>22.611177245508983</v>
       </c>
       <c r="R101" s="8">
-        <v>10.134543548387096</v>
+        <v>9.8377557823129251</v>
       </c>
       <c r="S101" s="8">
         <v>8</v>
       </c>
       <c r="T101" s="9">
-        <v>0.25</v>
+        <v>0.21556886227544911</v>
       </c>
       <c r="U101" s="9">
-        <v>0.40689655172413791</v>
+        <v>0.39644970414201186</v>
       </c>
       <c r="V101" s="9">
-        <v>0.089655172413793102</v>
+        <v>0.11242603550295859</v>
       </c>
       <c r="W101" s="9">
         <v>0</v>
       </c>
       <c r="X101" s="9">
-        <v>0.027586206896551724</v>
+        <v>0.023668639053254437</v>
       </c>
       <c r="Y101" s="9">
-        <v>0.020689655172413793</v>
+        <v>0.017751479289940829</v>
       </c>
       <c r="Z101" s="9">
-        <v>0.0068965517241379309</v>
+        <v>0.0059171597633136093</v>
       </c>
       <c r="AA101" s="9">
-        <v>0.15862068965517243</v>
+        <v>0.13609467455621302</v>
       </c>
       <c r="AB101" s="9">
-        <v>0.055172413793103448</v>
+        <v>0.047337278106508875</v>
       </c>
       <c r="AC101" s="9">
-        <v>0.13793103448275862</v>
+        <v>0.13017751479289941</v>
       </c>
       <c r="AD101" s="6">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="AE101" s="6">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="AF101" s="6">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="AG101" s="6">
         <v>0</v>
@@ -16692,7 +16689,7 @@
         <v>8</v>
       </c>
       <c r="AM101" s="6">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AN101" s="9">
         <v>0</v>
@@ -16897,7 +16894,7 @@
         <v>19754</v>
       </c>
       <c r="B103" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C103" s="4">
         <v>51</v>
@@ -16928,70 +16925,70 @@
       </c>
       <c r="L103" s="4"/>
       <c r="M103" s="5">
-        <v>61619.366666666676</v>
+        <v>66790.630000000005</v>
       </c>
       <c r="N103" s="6">
-        <v>527</v>
+        <v>673</v>
       </c>
       <c r="O103" s="6">
-        <v>305</v>
+        <v>392</v>
       </c>
       <c r="P103" s="7">
-        <v>2.547731379962193</v>
+        <v>2.5514747787610617</v>
       </c>
       <c r="Q103" s="8">
-        <v>15.558688852459015</v>
+        <v>15.842092091836733</v>
       </c>
       <c r="R103" s="8">
-        <v>4.9311950657894741</v>
+        <v>5.2410256410256411</v>
       </c>
       <c r="S103" s="8">
         <v>8</v>
       </c>
       <c r="T103" s="9">
-        <v>0.52131147540983602</v>
+        <v>0.50510204081632648</v>
       </c>
       <c r="U103" s="9">
-        <v>0.078688524590163941</v>
+        <v>0.091836734693877556</v>
       </c>
       <c r="V103" s="9">
-        <v>0.036065573770491806</v>
+        <v>0.03826530612244898</v>
       </c>
       <c r="W103" s="9">
         <v>0</v>
       </c>
       <c r="X103" s="9">
-        <v>0.029508196721311476</v>
+        <v>0.025510204081632654</v>
       </c>
       <c r="Y103" s="9">
         <v>0</v>
       </c>
       <c r="Z103" s="9">
-        <v>0.0032786885245901639</v>
+        <v>0.0025510204081632651</v>
       </c>
       <c r="AA103" s="9">
-        <v>0.0032786885245901639</v>
+        <v>0.0051020408163265302</v>
       </c>
       <c r="AB103" s="9">
-        <v>0.0098360655737704927</v>
+        <v>0.017857142857142856</v>
       </c>
       <c r="AC103" s="9">
-        <v>0</v>
+        <v>0.01020408163265306</v>
       </c>
       <c r="AD103" s="6">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="AE103" s="6">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="AF103" s="6">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AG103" s="6">
         <v>0</v>
       </c>
       <c r="AH103" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AI103" s="6">
         <v>0</v>
@@ -17000,13 +16997,13 @@
         <v>1</v>
       </c>
       <c r="AK103" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL103" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AM103" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AN103" s="9">
         <v>0</v>
@@ -18504,7 +18501,7 @@
         <v>321</v>
       </c>
       <c r="O113" s="6">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="P113" s="7">
         <v>6.2194273006134972</v>
@@ -18522,46 +18519,46 @@
         <v>0.2807017543859649</v>
       </c>
       <c r="U113" s="9">
-        <v>0.46721311475409838</v>
+        <v>0.36257309941520466</v>
       </c>
       <c r="V113" s="9">
-        <v>0.073770491803278687</v>
+        <v>0.058479532163742687</v>
       </c>
       <c r="W113" s="9">
-        <v>0.016393442622000001</v>
+        <v>0.011695906432000001</v>
       </c>
       <c r="X113" s="9">
-        <v>0.05737704918032787</v>
+        <v>0.058479532163742687</v>
       </c>
       <c r="Y113" s="9">
-        <v>0.049180327868852458</v>
+        <v>0.035087719298245612</v>
       </c>
       <c r="Z113" s="9">
         <v>0</v>
       </c>
       <c r="AA113" s="9">
-        <v>0.28688524590163933</v>
+        <v>0.21052631578947367</v>
       </c>
       <c r="AB113" s="9">
-        <v>0.0081967213114754103</v>
+        <v>0.0058479532163742687</v>
       </c>
       <c r="AC113" s="9">
-        <v>0.10655737704918032</v>
+        <v>0.076023391812865493</v>
       </c>
       <c r="AD113" s="6">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="AE113" s="6">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="AF113" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG113" s="6">
         <v>2</v>
       </c>
       <c r="AH113" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AI113" s="6">
         <v>6</v>
@@ -18570,7 +18567,7 @@
         <v>0</v>
       </c>
       <c r="AK113" s="6">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AL113" s="6">
         <v>1</v>
@@ -21419,7 +21416,7 @@
         <v>264</v>
       </c>
       <c r="O132" s="6">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="P132" s="7">
         <v>7.1985188888888896</v>
@@ -21437,7 +21434,7 @@
         <v>0.36021505376344087</v>
       </c>
       <c r="U132" s="9">
-        <v>0.2709677419354839</v>
+        <v>0.29569892473118281</v>
       </c>
       <c r="V132" s="9">
         <v>0</v>
@@ -21446,28 +21443,28 @@
         <v>0</v>
       </c>
       <c r="X132" s="9">
-        <v>0.051612903225806452</v>
+        <v>0.069892473118279563</v>
       </c>
       <c r="Y132" s="9">
-        <v>0.0064516129032258064</v>
+        <v>0.016129032258064516</v>
       </c>
       <c r="Z132" s="9">
         <v>0</v>
       </c>
       <c r="AA132" s="9">
-        <v>0.21935483870967742</v>
+        <v>0.23118279569892472</v>
       </c>
       <c r="AB132" s="9">
-        <v>0.01935483870967742</v>
+        <v>0.016129032258064516</v>
       </c>
       <c r="AC132" s="9">
-        <v>0.012903225806451613</v>
+        <v>0.010752688172043012</v>
       </c>
       <c r="AD132" s="6">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="AE132" s="6">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="AF132" s="6">
         <v>0</v>
@@ -21476,16 +21473,16 @@
         <v>0</v>
       </c>
       <c r="AH132" s="6">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AI132" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AJ132" s="6">
         <v>0</v>
       </c>
       <c r="AK132" s="6">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="AL132" s="6">
         <v>3</v>
@@ -24338,7 +24335,7 @@
         <v>274</v>
       </c>
       <c r="O151" s="6">
-        <v>67</v>
+        <v>235</v>
       </c>
       <c r="P151" s="7">
         <v>6.373504029304029</v>
@@ -24356,61 +24353,61 @@
         <v>0.28936170212765955</v>
       </c>
       <c r="U151" s="9">
-        <v>0.13432835820895522</v>
+        <v>0.18723404255319148</v>
       </c>
       <c r="V151" s="9">
-        <v>0.029850746268656716</v>
+        <v>0.034042553191489362</v>
       </c>
       <c r="W151" s="9">
         <v>0</v>
       </c>
       <c r="X151" s="9">
-        <v>0.014925373134328358</v>
+        <v>0.02553191489361702</v>
       </c>
       <c r="Y151" s="9">
-        <v>0</v>
+        <v>0.0042553191489361703</v>
       </c>
       <c r="Z151" s="9">
         <v>0</v>
       </c>
       <c r="AA151" s="9">
-        <v>0.014925373134328358</v>
+        <v>0.089361702127659579</v>
       </c>
       <c r="AB151" s="9">
-        <v>0.014925373134328358</v>
+        <v>0.01276595744680851</v>
       </c>
       <c r="AC151" s="9">
-        <v>0.059701492537313432</v>
+        <v>0.02553191489361702</v>
       </c>
       <c r="AD151" s="6">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="AE151" s="6">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="AF151" s="6">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AG151" s="6">
         <v>0</v>
       </c>
       <c r="AH151" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AI151" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ151" s="6">
         <v>0</v>
       </c>
       <c r="AK151" s="6">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="AL151" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM151" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN151" s="9">
         <v>0</v>
@@ -24772,7 +24769,7 @@
         <v>19898</v>
       </c>
       <c r="B154" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c t="s" r="C154" s="4">
         <v>51</v>
@@ -24801,88 +24798,88 @@
       </c>
       <c r="L154" s="4"/>
       <c r="M154" s="5">
-        <v>13522.32</v>
+        <v>15389.319999999998</v>
       </c>
       <c r="N154" s="6">
-        <v>89</v>
+        <v>184</v>
       </c>
       <c r="O154" s="6">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="P154" s="7">
-        <v>2.9956032967032966</v>
+        <v>3.4519752577319589</v>
       </c>
       <c r="Q154" s="8">
-        <v>16.260185185185183</v>
+        <v>19.926126126126128</v>
       </c>
       <c r="R154" s="8">
-        <v>6.6408792452830196</v>
+        <v>9.855351376146789</v>
       </c>
       <c r="S154" s="8">
         <v>7</v>
       </c>
       <c r="T154" s="9">
-        <v>0.55555555555555558</v>
+        <v>0.36036036036036034</v>
       </c>
       <c r="U154" s="9">
-        <v>0.18518518518518517</v>
+        <v>0.21621621621621623</v>
       </c>
       <c r="V154" s="9">
-        <v>0.07407407407407407</v>
+        <v>0.072072072072072071</v>
       </c>
       <c r="W154" s="9">
         <v>0</v>
       </c>
       <c r="X154" s="9">
-        <v>0.055555555555555552</v>
+        <v>0.036036036036036036</v>
       </c>
       <c r="Y154" s="9">
-        <v>0</v>
+        <v>0.0090090090090090089</v>
       </c>
       <c r="Z154" s="9">
         <v>0</v>
       </c>
       <c r="AA154" s="9">
-        <v>0.07407407407407407</v>
+        <v>0.045045045045045043</v>
       </c>
       <c r="AB154" s="9">
-        <v>0.018518518518518517</v>
+        <v>0.018018018018018018</v>
       </c>
       <c r="AC154" s="9">
-        <v>0</v>
+        <v>0.063063063063063057</v>
       </c>
       <c r="AD154" s="6">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="AE154" s="6">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="AF154" s="6">
+        <v>8</v>
+      </c>
+      <c r="AG154" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH154" s="6">
         <v>4</v>
       </c>
-      <c r="AG154" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH154" s="6">
-        <v>3</v>
-      </c>
       <c r="AI154" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ154" s="6">
         <v>0</v>
       </c>
       <c r="AK154" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL154" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM154" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AN154" s="9">
-        <v>0.018518518518518517</v>
+        <v>0.0090090090090090089</v>
       </c>
       <c r="AO154" s="6">
         <v>1</v>
@@ -25276,7 +25273,7 @@
         <v>587</v>
       </c>
       <c r="O157" s="6">
-        <v>195</v>
+        <v>283</v>
       </c>
       <c r="P157" s="7">
         <v>6.3254766031195846</v>
@@ -25294,25 +25291,25 @@
         <v>0.62190812720848054</v>
       </c>
       <c r="U157" s="9">
-        <v>0.030769230769230771</v>
+        <v>0.021201413427561839</v>
       </c>
       <c r="V157" s="9">
-        <v>0.0051282051282051282</v>
+        <v>0.0035335689045936395</v>
       </c>
       <c r="W157" s="9">
         <v>0</v>
       </c>
       <c r="X157" s="9">
-        <v>0.02564102564102564</v>
+        <v>0.017667844522968199</v>
       </c>
       <c r="Y157" s="9">
-        <v>0.0051282051282051282</v>
+        <v>0.0035335689045936395</v>
       </c>
       <c r="Z157" s="9">
         <v>0</v>
       </c>
       <c r="AA157" s="9">
-        <v>0.0051282051282051282</v>
+        <v>0.0035335689045936395</v>
       </c>
       <c r="AB157" s="9">
         <v>0</v>
@@ -26592,7 +26589,7 @@
         <v>19927</v>
       </c>
       <c r="B166" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C166" s="4">
         <v>51</v>
@@ -26623,34 +26620,34 @@
       </c>
       <c r="L166" s="4"/>
       <c r="M166" s="5">
-        <v>10608.196666666667</v>
+        <v>12048.09</v>
       </c>
       <c r="N166" s="6">
-        <v>122</v>
+        <v>160</v>
       </c>
       <c r="O166" s="6">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="P166" s="7">
-        <v>7.4154572580645164</v>
+        <v>8.5958079754601222</v>
       </c>
       <c r="Q166" s="8">
-        <v>22.433146067415731</v>
+        <v>24.063498347107441</v>
       </c>
       <c r="R166" s="8">
-        <v>8.781418390804598</v>
+        <v>9.1209410256410255</v>
       </c>
       <c r="S166" s="8">
         <v>7</v>
       </c>
       <c r="T166" s="9">
-        <v>0.15730337078651685</v>
+        <v>0.14049586776859505</v>
       </c>
       <c r="U166" s="9">
-        <v>0.10112359550561797</v>
+        <v>0.13223140495867769</v>
       </c>
       <c r="V166" s="9">
-        <v>0.078651685393258425</v>
+        <v>0.082644628099173556</v>
       </c>
       <c r="W166" s="9">
         <v>0</v>
@@ -26665,22 +26662,22 @@
         <v>0</v>
       </c>
       <c r="AA166" s="9">
-        <v>0.02247191011235955</v>
+        <v>0.033057851239669422</v>
       </c>
       <c r="AB166" s="9">
-        <v>0</v>
+        <v>0.016528925619834711</v>
       </c>
       <c r="AC166" s="9">
         <v>0</v>
       </c>
       <c r="AD166" s="6">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AE166" s="6">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AF166" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AG166" s="6">
         <v>0</v>
@@ -26695,10 +26692,10 @@
         <v>0</v>
       </c>
       <c r="AK166" s="6">
+        <v>4</v>
+      </c>
+      <c r="AL166" s="6">
         <v>2</v>
-      </c>
-      <c r="AL166" s="6">
-        <v>0</v>
       </c>
       <c r="AM166" s="6">
         <v>0</v>
@@ -26749,7 +26746,7 @@
         <v>19928</v>
       </c>
       <c r="B167" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C167" s="4">
         <v>51</v>
@@ -26780,85 +26777,85 @@
       </c>
       <c r="L167" s="4"/>
       <c r="M167" s="5">
-        <v>26917.800000000003</v>
+        <v>27814.060000000001</v>
       </c>
       <c r="N167" s="6">
-        <v>263</v>
+        <v>317</v>
       </c>
       <c r="O167" s="6">
-        <v>186</v>
+        <v>230</v>
       </c>
       <c r="P167" s="7">
-        <v>5.1864620689655174</v>
+        <v>4.9053268987341774</v>
       </c>
       <c r="Q167" s="8">
-        <v>18.707706451612903</v>
+        <v>17.65565260869565</v>
       </c>
       <c r="R167" s="8">
-        <v>7.6579545454545448</v>
+        <v>6.8995348837209303</v>
       </c>
       <c r="S167" s="8">
         <v>7</v>
       </c>
       <c r="T167" s="9">
-        <v>0.44086021505376344</v>
+        <v>0.4826086956521739</v>
       </c>
       <c r="U167" s="9">
-        <v>0.25268817204301075</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="V167" s="9">
-        <v>0.016129032258064516</v>
+        <v>0.017391304347826087</v>
       </c>
       <c r="W167" s="9">
         <v>0</v>
       </c>
       <c r="X167" s="9">
-        <v>0.075268817204301078</v>
+        <v>0.069565217391304349</v>
       </c>
       <c r="Y167" s="9">
-        <v>0.010752688172043012</v>
+        <v>0.017391304347826087</v>
       </c>
       <c r="Z167" s="9">
         <v>0</v>
       </c>
       <c r="AA167" s="9">
-        <v>0.075268817204301078</v>
+        <v>0.091304347826086957</v>
       </c>
       <c r="AB167" s="9">
-        <v>0.043010752688172046</v>
+        <v>0.039130434782608699</v>
       </c>
       <c r="AC167" s="9">
-        <v>0.086021505376344093</v>
+        <v>0.095652173913043481</v>
       </c>
       <c r="AD167" s="6">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="AE167" s="6">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="AF167" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG167" s="6">
         <v>0</v>
       </c>
       <c r="AH167" s="6">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AI167" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AJ167" s="6">
         <v>0</v>
       </c>
       <c r="AK167" s="6">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="AL167" s="6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AM167" s="6">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="AN167" s="9">
         <v>0</v>
@@ -26906,7 +26903,7 @@
         <v>19930</v>
       </c>
       <c r="B168" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C168" s="4">
         <v>51</v>
@@ -26937,40 +26934,40 @@
       </c>
       <c r="L168" s="4"/>
       <c r="M168" s="5">
-        <v>31574.64333333333</v>
+        <v>34377.979999999996</v>
       </c>
       <c r="N168" s="6">
-        <v>337</v>
+        <v>422</v>
       </c>
       <c r="O168" s="6">
-        <v>267</v>
+        <v>340</v>
       </c>
       <c r="P168" s="7">
-        <v>4.3374631268436579</v>
+        <v>4.4237983451536644</v>
       </c>
       <c r="Q168" s="8">
-        <v>21.61654194756554</v>
+        <v>21.392598235294116</v>
       </c>
       <c r="R168" s="8">
-        <v>10.639330681818182</v>
+        <v>10.24272997032641</v>
       </c>
       <c r="S168" s="8">
         <v>7</v>
       </c>
       <c r="T168" s="9">
-        <v>0.16104868913857678</v>
+        <v>0.14411764705882352</v>
       </c>
       <c r="U168" s="9">
-        <v>0.25093632958801498</v>
+        <v>0.22941176470588234</v>
       </c>
       <c r="V168" s="9">
-        <v>0.014981273408239701</v>
+        <v>0.011764705882352941</v>
       </c>
       <c r="W168" s="9">
         <v>0</v>
       </c>
       <c r="X168" s="9">
-        <v>0.037453183520599252</v>
+        <v>0.032352941176470591</v>
       </c>
       <c r="Y168" s="9">
         <v>0</v>
@@ -26979,19 +26976,19 @@
         <v>0</v>
       </c>
       <c r="AA168" s="9">
-        <v>0.011235955056179775</v>
+        <v>0.0088235294117647058</v>
       </c>
       <c r="AB168" s="9">
-        <v>0.0074906367041198503</v>
+        <v>0.011764705882352941</v>
       </c>
       <c r="AC168" s="9">
-        <v>0.18352059925093633</v>
+        <v>0.1676470588235294</v>
       </c>
       <c r="AD168" s="6">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="AE168" s="6">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="AF168" s="6">
         <v>4</v>
@@ -27000,7 +26997,7 @@
         <v>0</v>
       </c>
       <c r="AH168" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AI168" s="6">
         <v>0</v>
@@ -27012,10 +27009,10 @@
         <v>3</v>
       </c>
       <c r="AL168" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AM168" s="6">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="AN168" s="9">
         <v>0</v>
@@ -27063,7 +27060,7 @@
         <v>19931</v>
       </c>
       <c r="B169" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C169" s="4">
         <v>51</v>
@@ -27094,85 +27091,85 @@
       </c>
       <c r="L169" s="4"/>
       <c r="M169" s="5">
-        <v>28476.746666666662</v>
+        <v>34695.910000000003</v>
       </c>
       <c r="N169" s="6">
-        <v>280</v>
+        <v>388</v>
       </c>
       <c r="O169" s="6">
-        <v>104</v>
+        <v>153</v>
       </c>
       <c r="P169" s="7">
-        <v>4.5436512820512815</v>
+        <v>4.5624348167539273</v>
       </c>
       <c r="Q169" s="8">
-        <v>15.745351923076923</v>
+        <v>15.975381045751632</v>
       </c>
       <c r="R169" s="8">
-        <v>4.3039916666666667</v>
+        <v>4.515267132867133</v>
       </c>
       <c r="S169" s="8">
         <v>7</v>
       </c>
       <c r="T169" s="9">
-        <v>0.51923076923076927</v>
+        <v>0.47712418300653597</v>
       </c>
       <c r="U169" s="9">
-        <v>0.19230769230769232</v>
+        <v>0.18300653594771241</v>
       </c>
       <c r="V169" s="9">
-        <v>0.019230769230769232</v>
+        <v>0.019607843137254902</v>
       </c>
       <c r="W169" s="9">
         <v>0</v>
       </c>
       <c r="X169" s="9">
-        <v>0.11538461538461539</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="Y169" s="9">
-        <v>0.028846153846153848</v>
+        <v>0.032679738562091505</v>
       </c>
       <c r="Z169" s="9">
         <v>0</v>
       </c>
       <c r="AA169" s="9">
-        <v>0.11538461538461539</v>
+        <v>0.091503267973856203</v>
       </c>
       <c r="AB169" s="9">
-        <v>0.019230769230769232</v>
+        <v>0.026143790849673203</v>
       </c>
       <c r="AC169" s="9">
-        <v>0</v>
+        <v>0.013071895424836602</v>
       </c>
       <c r="AD169" s="6">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="AE169" s="6">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="AF169" s="6">
+        <v>3</v>
+      </c>
+      <c r="AG169" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH169" s="6">
+        <v>17</v>
+      </c>
+      <c r="AI169" s="6">
+        <v>5</v>
+      </c>
+      <c r="AJ169" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK169" s="6">
+        <v>14</v>
+      </c>
+      <c r="AL169" s="6">
+        <v>4</v>
+      </c>
+      <c r="AM169" s="6">
         <v>2</v>
-      </c>
-      <c r="AG169" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH169" s="6">
-        <v>12</v>
-      </c>
-      <c r="AI169" s="6">
-        <v>3</v>
-      </c>
-      <c r="AJ169" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK169" s="6">
-        <v>12</v>
-      </c>
-      <c r="AL169" s="6">
-        <v>2</v>
-      </c>
-      <c r="AM169" s="6">
-        <v>0</v>
       </c>
       <c r="AN169" s="9">
         <v>0</v>
@@ -27689,7 +27686,7 @@
         <v>19943</v>
       </c>
       <c r="B173" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C173" s="4">
         <v>51</v>
@@ -27720,55 +27717,55 @@
       </c>
       <c r="L173" s="4"/>
       <c r="M173" s="5">
-        <v>17475.710000000003</v>
+        <v>18915.139999999996</v>
       </c>
       <c r="N173" s="6">
-        <v>190</v>
+        <v>237</v>
       </c>
       <c r="O173" s="6">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="P173" s="7">
-        <v>7.7055845744680846</v>
+        <v>7.4994323404255319</v>
       </c>
       <c r="Q173" s="8">
-        <v>19.814833027522937</v>
+        <v>20.07676893939394</v>
       </c>
       <c r="R173" s="8">
-        <v>6.8063504761904756</v>
+        <v>7.0165375000000001</v>
       </c>
       <c r="S173" s="8">
         <v>7</v>
       </c>
       <c r="T173" s="9">
-        <v>0.26605504587155965</v>
+        <v>0.24242424242424243</v>
       </c>
       <c r="U173" s="9">
-        <v>0.15596330275229359</v>
+        <v>0.12878787878787878</v>
       </c>
       <c r="V173" s="9">
-        <v>0.01834862385321101</v>
+        <v>0.015151515151515152</v>
       </c>
       <c r="W173" s="9">
         <v>0</v>
       </c>
       <c r="X173" s="9">
-        <v>0.082568807339449546</v>
+        <v>0.068181818181818177</v>
       </c>
       <c r="Y173" s="9">
-        <v>0.01834862385321101</v>
+        <v>0.015151515151515152</v>
       </c>
       <c r="Z173" s="9">
-        <v>0.0091743119266055051</v>
+        <v>0.007575757575757576</v>
       </c>
       <c r="AA173" s="9">
-        <v>0.045871559633027525</v>
+        <v>0.03787878787878788</v>
       </c>
       <c r="AB173" s="9">
-        <v>0.01834862385321101</v>
+        <v>0.015151515151515152</v>
       </c>
       <c r="AC173" s="9">
-        <v>0.01834862385321101</v>
+        <v>0.015151515151515152</v>
       </c>
       <c r="AD173" s="6">
         <v>23</v>
@@ -28631,7 +28628,7 @@
         <v>19954</v>
       </c>
       <c r="B179" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C179" s="4">
         <v>51</v>
@@ -28662,40 +28659,40 @@
       </c>
       <c r="L179" s="4"/>
       <c r="M179" s="5">
-        <v>11691.528333333335</v>
+        <v>15001.980000000001</v>
       </c>
       <c r="N179" s="6">
-        <v>129</v>
+        <v>193</v>
       </c>
       <c r="O179" s="6">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="P179" s="7">
-        <v>6.7216148437500003</v>
+        <v>7.7970489583333338</v>
       </c>
       <c r="Q179" s="8">
-        <v>18.122805263157897</v>
+        <v>18.628276404494382</v>
       </c>
       <c r="R179" s="8">
-        <v>3.9856719298245613</v>
+        <v>4.1503741573033714</v>
       </c>
       <c r="S179" s="8">
         <v>7</v>
       </c>
       <c r="T179" s="9">
-        <v>0.45614035087719296</v>
+        <v>0.43820224719101125</v>
       </c>
       <c r="U179" s="9">
-        <v>0.08771929824561403</v>
+        <v>0.0898876404494382</v>
       </c>
       <c r="V179" s="9">
-        <v>0.070175438596491224</v>
+        <v>0.056179775280898875</v>
       </c>
       <c r="W179" s="9">
-        <v>0.017543859649000001</v>
+        <v>0.011235955056</v>
       </c>
       <c r="X179" s="9">
-        <v>0.035087719298245612</v>
+        <v>0.033707865168539325</v>
       </c>
       <c r="Y179" s="9">
         <v>0</v>
@@ -28704,28 +28701,28 @@
         <v>0</v>
       </c>
       <c r="AA179" s="9">
-        <v>0</v>
+        <v>0.011235955056179775</v>
       </c>
       <c r="AB179" s="9">
-        <v>0.017543859649122806</v>
+        <v>0.011235955056179775</v>
       </c>
       <c r="AC179" s="9">
         <v>0</v>
       </c>
       <c r="AD179" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AE179" s="6">
+        <v>8</v>
+      </c>
+      <c r="AF179" s="6">
         <v>5</v>
       </c>
-      <c r="AF179" s="6">
-        <v>4</v>
-      </c>
       <c r="AG179" s="6">
         <v>1</v>
       </c>
       <c r="AH179" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI179" s="6">
         <v>0</v>
@@ -28734,7 +28731,7 @@
         <v>0</v>
       </c>
       <c r="AK179" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL179" s="6">
         <v>1</v>
@@ -29102,7 +29099,7 @@
         <v>19959</v>
       </c>
       <c r="B182" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C182" s="4">
         <v>51</v>
@@ -29133,40 +29130,40 @@
       </c>
       <c r="L182" s="4"/>
       <c r="M182" s="5">
-        <v>14748.125</v>
+        <v>18255.450000000001</v>
       </c>
       <c r="N182" s="6">
-        <v>148</v>
+        <v>204</v>
       </c>
       <c r="O182" s="6">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="P182" s="7">
-        <v>4.9819156028368798</v>
+        <v>5.649830612244898</v>
       </c>
       <c r="Q182" s="8">
-        <v>16.967968750000001</v>
+        <v>16.642181481481479</v>
       </c>
       <c r="R182" s="8">
-        <v>5.2502650793650796</v>
+        <v>4.6919835443037972</v>
       </c>
       <c r="S182" s="8">
         <v>7</v>
       </c>
       <c r="T182" s="9">
-        <v>0.46875</v>
+        <v>0.49382716049382713</v>
       </c>
       <c r="U182" s="9">
-        <v>0.15625</v>
+        <v>0.16049382716049382</v>
       </c>
       <c r="V182" s="9">
-        <v>0.078125</v>
+        <v>0.07407407407407407</v>
       </c>
       <c r="W182" s="9">
         <v>0</v>
       </c>
       <c r="X182" s="9">
-        <v>0</v>
+        <v>0.012345679012345678</v>
       </c>
       <c r="Y182" s="9">
         <v>0</v>
@@ -29175,37 +29172,37 @@
         <v>0</v>
       </c>
       <c r="AA182" s="9">
-        <v>0.046875</v>
+        <v>0.061728395061728392</v>
       </c>
       <c r="AB182" s="9">
-        <v>0.03125</v>
+        <v>0.024691358024691357</v>
       </c>
       <c r="AC182" s="9">
         <v>0</v>
       </c>
       <c r="AD182" s="6">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="AE182" s="6">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AF182" s="6">
+        <v>6</v>
+      </c>
+      <c r="AG182" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH182" s="6">
+        <v>1</v>
+      </c>
+      <c r="AI182" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ182" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK182" s="6">
         <v>5</v>
-      </c>
-      <c r="AG182" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH182" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI182" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ182" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK182" s="6">
-        <v>3</v>
       </c>
       <c r="AL182" s="6">
         <v>2</v>
@@ -29259,7 +29256,7 @@
         <v>19961</v>
       </c>
       <c r="B183" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C183" s="4">
         <v>51</v>
@@ -29290,82 +29287,82 @@
       </c>
       <c r="L183" s="4"/>
       <c r="M183" s="5">
-        <v>18499.063333333335</v>
+        <v>20894.170000000002</v>
       </c>
       <c r="N183" s="6">
-        <v>179</v>
+        <v>230</v>
       </c>
       <c r="O183" s="6">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="P183" s="7">
-        <v>6.1321833333333338</v>
+        <v>6.0183031250000001</v>
       </c>
       <c r="Q183" s="8">
-        <v>16.492095876288662</v>
+        <v>16.221774193548388</v>
       </c>
       <c r="R183" s="8">
-        <v>3.3527173913043478</v>
+        <v>3.4462965811965813</v>
       </c>
       <c r="S183" s="8">
         <v>7</v>
       </c>
       <c r="T183" s="9">
-        <v>0.46391752577319589</v>
+        <v>0.45967741935483869</v>
       </c>
       <c r="U183" s="9">
-        <v>0.14432989690721648</v>
+        <v>0.16129032258064516</v>
       </c>
       <c r="V183" s="9">
-        <v>0.010309278350515464</v>
+        <v>0.024193548387096774</v>
       </c>
       <c r="W183" s="9">
         <v>0</v>
       </c>
       <c r="X183" s="9">
-        <v>0.020618556701030927</v>
+        <v>0.024193548387096774</v>
       </c>
       <c r="Y183" s="9">
-        <v>0.010309278350515464</v>
+        <v>0.016129032258064516</v>
       </c>
       <c r="Z183" s="9">
-        <v>0.010309278350515464</v>
+        <v>0.0080645161290322578</v>
       </c>
       <c r="AA183" s="9">
-        <v>0.08247422680412371</v>
+        <v>0.096774193548387094</v>
       </c>
       <c r="AB183" s="9">
-        <v>0.030927835051546393</v>
+        <v>0.032258064516129031</v>
       </c>
       <c r="AC183" s="9">
-        <v>0.020618556701030927</v>
+        <v>0.016129032258064516</v>
       </c>
       <c r="AD183" s="6">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="AE183" s="6">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="AF183" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG183" s="6">
         <v>0</v>
       </c>
       <c r="AH183" s="6">
+        <v>3</v>
+      </c>
+      <c r="AI183" s="6">
         <v>2</v>
       </c>
-      <c r="AI183" s="6">
-        <v>1</v>
-      </c>
       <c r="AJ183" s="6">
         <v>1</v>
       </c>
       <c r="AK183" s="6">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AL183" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AM183" s="6">
         <v>2</v>
@@ -30137,52 +30134,52 @@
         <v>312</v>
       </c>
       <c t="s" r="Z189" s="11">
+        <v>310</v>
+      </c>
+      <c t="s" r="AA189" s="11">
         <v>313</v>
       </c>
-      <c t="s" r="AA189" s="11">
+      <c t="s" r="AB189" s="11">
         <v>314</v>
       </c>
-      <c t="s" r="AB189" s="11">
+      <c t="s" r="AC189" s="11">
         <v>315</v>
       </c>
-      <c t="s" r="AC189" s="11">
+      <c t="s" r="AD189" s="11">
         <v>316</v>
       </c>
-      <c t="s" r="AD189" s="11">
+      <c t="s" r="AE189" s="11">
         <v>317</v>
       </c>
-      <c t="s" r="AE189" s="11">
+      <c t="s" r="AF189" s="11">
         <v>318</v>
       </c>
-      <c t="s" r="AF189" s="11">
+      <c t="s" r="AG189" s="11">
         <v>319</v>
       </c>
-      <c t="s" r="AG189" s="11">
+      <c t="s" r="AH189" s="11">
         <v>320</v>
       </c>
-      <c t="s" r="AH189" s="11">
+      <c t="s" r="AI189" s="11">
         <v>321</v>
       </c>
-      <c t="s" r="AI189" s="11">
+      <c t="s" r="AJ189" s="11">
         <v>322</v>
       </c>
-      <c t="s" r="AJ189" s="11">
+      <c t="s" r="AK189" s="11">
         <v>323</v>
       </c>
-      <c t="s" r="AK189" s="11">
+      <c t="s" r="AL189" s="11">
         <v>324</v>
       </c>
-      <c t="s" r="AL189" s="11">
+      <c t="s" r="AM189" s="11">
         <v>325</v>
       </c>
-      <c t="s" r="AM189" s="11">
+      <c t="s" r="AN189" s="11">
         <v>326</v>
       </c>
-      <c t="s" r="AN189" s="11">
+      <c t="s" r="AO189" s="11">
         <v>327</v>
-      </c>
-      <c t="s" r="AO189" s="11">
-        <v>328</v>
       </c>
       <c r="AP189" s="12"/>
       <c t="s" r="AQ189" s="12">
@@ -30199,10 +30196,10 @@
         <v>59</v>
       </c>
       <c t="s" r="AX189" s="11">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c t="s" r="AY189" s="11">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AZ189" s="12"/>
       <c r="BA189" s="12"/>

</xml_diff>